<commit_message>
Add Kinnan activation cost reduction support
</commit_message>
<xml_diff>
--- a/reports/kinnan_100/experiment.xlsx
+++ b/reports/kinnan_100/experiment.xlsx
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>36</v>
+        <v>58</v>
       </c>
     </row>
     <row r="20">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>0.36</v>
+        <v>0.58</v>
       </c>
     </row>
     <row r="21">
@@ -882,7 +882,7 @@
         <v>6</v>
       </c>
       <c r="C8" s="9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D8" s="9" t="b">
         <v>1</v>
@@ -990,7 +990,7 @@
         <v>6</v>
       </c>
       <c r="C14" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D14" s="9" t="b">
         <v>1</v>
@@ -1026,7 +1026,7 @@
         <v>6</v>
       </c>
       <c r="C16" s="9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D16" s="9" t="b">
         <v>1</v>
@@ -1062,7 +1062,7 @@
         <v>6</v>
       </c>
       <c r="C18" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D18" s="9" t="b">
         <v>1</v>
@@ -1134,7 +1134,7 @@
         <v>6</v>
       </c>
       <c r="C22" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D22" s="9" t="b">
         <v>1</v>
@@ -1170,7 +1170,7 @@
         <v>6</v>
       </c>
       <c r="C24" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D24" s="9" t="b">
         <v>1</v>
@@ -1422,7 +1422,7 @@
         <v>6</v>
       </c>
       <c r="C38" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D38" s="9" t="b">
         <v>1</v>
@@ -1566,7 +1566,7 @@
         <v>6</v>
       </c>
       <c r="C46" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D46" s="9" t="b">
         <v>1</v>
@@ -1620,7 +1620,7 @@
         <v>6</v>
       </c>
       <c r="C49" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D49" s="9" t="b">
         <v>1</v>
@@ -1656,7 +1656,7 @@
         <v>6</v>
       </c>
       <c r="C51" s="9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D51" s="9" t="b">
         <v>1</v>
@@ -1728,7 +1728,7 @@
         <v>6</v>
       </c>
       <c r="C55" s="9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D55" s="9" t="b">
         <v>1</v>
@@ -1908,7 +1908,7 @@
         <v>6</v>
       </c>
       <c r="C65" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D65" s="9" t="b">
         <v>1</v>
@@ -1944,7 +1944,7 @@
         <v>6</v>
       </c>
       <c r="C67" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D67" s="9" t="b">
         <v>1</v>
@@ -2178,7 +2178,7 @@
         <v>6</v>
       </c>
       <c r="C80" s="9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D80" s="9" t="b">
         <v>1</v>
@@ -2412,7 +2412,7 @@
         <v>6</v>
       </c>
       <c r="C93" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D93" s="9" t="b">
         <v>1</v>
@@ -2466,7 +2466,7 @@
         <v>6</v>
       </c>
       <c r="C96" s="9" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D96" s="9" t="b">
         <v>1</v>

</xml_diff>